<commit_message>
Major changes in working hours and hardruling in same driver not asigning 2 vehicles at sametime
</commit_message>
<xml_diff>
--- a/PLANNED.xlsx
+++ b/PLANNED.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FleetPlanner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46ED8F3C-B20B-43D9-9C94-DEFFE5D64004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5DC0E75-0994-4959-92AF-CCFBD181D8E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="237">
   <si>
     <r>
       <rPr>
@@ -143,16 +143,6 @@
         <family val="2"/>
       </rPr>
       <t>VEHICLE</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>DRIVER</t>
     </r>
   </si>
   <si>
@@ -256,26 +246,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>P 29760</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>ARAVIND BALAKRISHNAN</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>162822
 (1628221)</t>
     </r>
@@ -368,6 +338,17 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
+      <t>601928 - 601928 - Apartment Club
+2026</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial MT"/>
+        <family val="2"/>
+      </rPr>
       <t>5 Ton Chiller Truck (with lift)</t>
     </r>
   </si>
@@ -379,26 +360,6 @@
         <family val="2"/>
       </rPr>
       <t>APPARTMENT CLUB MORNING BREAKFAST PICK UP @ 6:00AM FOR THE MONTH OF FEB 2026</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>B 50741</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>SHIB BAHADUR</t>
     </r>
   </si>
   <si>
@@ -500,26 +461,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>B 50368</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>DEEPAK DEWAN</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>162779
 (1627791)</t>
     </r>
@@ -531,16 +472,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>07:00 - 11:00</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>SUMON - 0561165608</t>
     </r>
   </si>
@@ -706,38 +637,7 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>4.2 Ton Double cabin Open Truck
-(with lift)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>TO BRING EQUIPMENT FROM JWH</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>Z 43915</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>KARIM KHAN</t>
     </r>
   </si>
   <si>
@@ -758,16 +658,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>09:00 - 17:00</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>UNNI - 0507101850</t>
     </r>
   </si>
@@ -827,26 +717,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>D 66528</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>RAMIL ANCHETA MANALO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>162473
 (1624731)</t>
     </r>
@@ -858,16 +728,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>09:00 - 13:00</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>CPK ONLY</t>
     </r>
   </si>
@@ -1019,16 +879,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>T 82656</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>162641
 (1626412)</t>
     </r>
@@ -1235,26 +1085,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>T 82659</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>VISWANADHAN</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>162785
 (1627851)</t>
     </r>
@@ -1358,26 +1188,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>A 67338</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>AALIM HASSAN</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>162787
 (1627871)</t>
     </r>
@@ -1420,16 +1230,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>13:00 - 20:00</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t xml:space="preserve">Arab Hope makers event on 13th, 14th, 15th Feb 2026 in Dubai ( coca cola Arena ) - FOOD PICK UP @1PM - </t>
     </r>
     <r>
@@ -1458,16 +1258,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>13:00 - 17:00</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>THOMAS - 0506884761</t>
     </r>
   </si>
@@ -1528,26 +1318,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>B 51850</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>IMRAN PASHA</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>162799
 (1627991)</t>
     </r>
@@ -1589,26 +1359,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>AA 16433</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>RASHEED THANDAPPURAM</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>162776
 (1627761)</t>
     </r>
@@ -1834,26 +1584,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>A 68982</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>MANPREET SINGH</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>161459
 (1614591)</t>
     </r>
@@ -2030,16 +1760,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>16:00 - 18:00</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>11 STAFF TRANSPORTATION</t>
     </r>
   </si>
@@ -2061,16 +1781,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>16:00 - 21:00</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>ONSITE - MENA PORT RASHID</t>
     </r>
   </si>
@@ -2102,16 +1812,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>16:00 - 19:00</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>ONSITE - DCRC AL MARMOUM</t>
     </r>
   </si>
@@ -2204,16 +1904,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>I 72610</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>162546
 (1625461)</t>
     </r>
@@ -2297,27 +1987,7 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>22:00 - 04:00</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>DINNER CLEARANCE + STAFF PICKUP</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
-      <t>D 18572</t>
     </r>
   </si>
   <si>
@@ -2369,16 +2039,6 @@
         <rFont val="Arial MT"/>
         <family val="2"/>
       </rPr>
-      <t>23:00 - 05:00</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial MT"/>
-        <family val="2"/>
-      </rPr>
       <t>ON SITE - PALM JUMEIRAH</t>
     </r>
   </si>
@@ -2477,47 +2137,155 @@
     </r>
   </si>
   <si>
+    <t>20 Seater Bus</t>
+  </si>
+  <si>
+    <t>23 Seater Bus</t>
+  </si>
+  <si>
+    <t>14 Seater Bus</t>
+  </si>
+  <si>
+    <t>5 Ton Chiller Truck (with lift)</t>
+  </si>
+  <si>
+    <t>5 Ton DryTruck (with lift)</t>
+  </si>
+  <si>
+    <t>5 Ton Open Truck (with lift)</t>
+  </si>
+  <si>
+    <t>12:00 - 13:00</t>
+  </si>
+  <si>
+    <t>13:00 - 15:00</t>
+  </si>
+  <si>
+    <t>15:00 - 17:00</t>
+  </si>
+  <si>
+    <t>07:00 - 09:00</t>
+  </si>
+  <si>
+    <t>16:00 - 17:00</t>
+  </si>
+  <si>
+    <t>Same Driver</t>
+  </si>
+  <si>
+    <t>P 29760</t>
+  </si>
+  <si>
+    <t>ARAVIND BALAKRISHNAN</t>
+  </si>
+  <si>
+    <t>B 50741</t>
+  </si>
+  <si>
+    <t>SHIB BAHADUR</t>
+  </si>
+  <si>
+    <t>07:00 - 15:00</t>
+  </si>
+  <si>
+    <t>B 50368</t>
+  </si>
+  <si>
+    <t>DEEPAK DEWAN</t>
+  </si>
+  <si>
+    <t>Z 43915</t>
+  </si>
+  <si>
+    <t>KARIM KHAN</t>
+  </si>
+  <si>
+    <t>D 66528</t>
+  </si>
+  <si>
+    <t>RAMIL ANCHETA MANALO</t>
+  </si>
+  <si>
+    <t>T 82656</t>
+  </si>
+  <si>
     <t>MUHAMMAD ATIF</t>
   </si>
   <si>
-    <t>20 Seater Bus</t>
-  </si>
-  <si>
-    <t>23 Seater Bus</t>
-  </si>
-  <si>
-    <t>14 Seater Bus</t>
-  </si>
-  <si>
-    <t>5 Ton Chiller Truck (with lift)</t>
-  </si>
-  <si>
-    <t>5 Ton DryTruck (with lift)</t>
-  </si>
-  <si>
-    <t>5 Ton Open Truck (with lift)</t>
-  </si>
-  <si>
-    <t>12:00 - 13:00</t>
-  </si>
-  <si>
-    <t>13:00 - 15:00</t>
-  </si>
-  <si>
-    <t>15:00 - 17:00</t>
-  </si>
-  <si>
-    <t>07:00 - 09:00</t>
-  </si>
-  <si>
-    <t>16:00 - 17:00</t>
-  </si>
-  <si>
-    <t>Same Driver</t>
-  </si>
-  <si>
-    <t>601928 - 601928 - Apartment Club
-2026</t>
+    <t>T 82659</t>
+  </si>
+  <si>
+    <t>VISWANADHAN</t>
+  </si>
+  <si>
+    <t>A 67338</t>
+  </si>
+  <si>
+    <t>AALIM HASSAN</t>
+  </si>
+  <si>
+    <t>B 51850</t>
+  </si>
+  <si>
+    <t>IMRAN PASHA</t>
+  </si>
+  <si>
+    <t>AA 16433</t>
+  </si>
+  <si>
+    <t>RASHEED THANDAPPURAM</t>
+  </si>
+  <si>
+    <t>A 68982</t>
+  </si>
+  <si>
+    <t>MANPREET SINGH</t>
+  </si>
+  <si>
+    <t>16:00 - 19:00</t>
+  </si>
+  <si>
+    <t>I 72610</t>
+  </si>
+  <si>
+    <t>D 18572</t>
+  </si>
+  <si>
+    <t>23:00 - 00:00</t>
+  </si>
+  <si>
+    <t>13:00 - 16:00</t>
+  </si>
+  <si>
+    <t>23:00 - 01:00</t>
+  </si>
+  <si>
+    <t>DRIVER</t>
+  </si>
+  <si>
+    <t>23:00 - 02:00</t>
+  </si>
+  <si>
+    <t>17:00 - 20:00</t>
+  </si>
+  <si>
+    <t>09:00 - 18:00</t>
+  </si>
+  <si>
+    <t>22:00 - 01:00</t>
+  </si>
+  <si>
+    <t>10:00 - 13:00</t>
+  </si>
+  <si>
+    <t>17:00 - 18:00</t>
+  </si>
+  <si>
+    <t>22:00 - 23:00</t>
+  </si>
+  <si>
+    <t>4.2 Ton Double cabin Open Truck 
+(with lift)</t>
   </si>
 </sst>
 </file>
@@ -2527,7 +2295,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy;@"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -2573,6 +2341,13 @@
       <color rgb="FFFFFF00"/>
       <name val="Arial MT"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="11">
@@ -2655,7 +2430,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -2708,6 +2483,12 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3014,7 +2795,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A581A1F3-CAF0-45C6-9B1F-97A2BD6208C7}">
-  <dimension ref="A1:N45"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:N47"/>
   <sheetFormatPr defaultRowHeight="10.199999999999999"/>
   <cols>
     <col min="1" max="1" width="6.44140625" style="15" customWidth="1"/>
@@ -3025,10 +2807,11 @@
     <col min="6" max="6" width="11.77734375" style="15" customWidth="1"/>
     <col min="7" max="7" width="14" style="15" customWidth="1"/>
     <col min="8" max="8" width="28.109375" style="15" customWidth="1"/>
-    <col min="9" max="9" width="23" style="16" customWidth="1"/>
+    <col min="9" max="9" width="18" style="16" customWidth="1"/>
     <col min="10" max="10" width="39.6640625" style="15" customWidth="1"/>
     <col min="11" max="11" width="8.88671875" style="15"/>
-    <col min="12" max="13" width="17.44140625" style="15" customWidth="1"/>
+    <col min="12" max="12" width="17.44140625" style="15" customWidth="1"/>
+    <col min="13" max="13" width="27.109375" style="15" customWidth="1"/>
     <col min="14" max="16384" width="8.88671875" style="15"/>
   </cols>
   <sheetData>
@@ -3066,317 +2849,317 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="19" t="s">
+        <v>228</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>12</v>
-      </c>
     </row>
-    <row r="2" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="2" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A2" s="3">
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C2" s="5">
         <v>46068</v>
       </c>
       <c r="D2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="H2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="I2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="J2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="4" t="s">
-        <v>20</v>
-      </c>
       <c r="K2" s="6" t="s">
-        <v>21</v>
+        <v>199</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>22</v>
+        <v>200</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="N2" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="3" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="3" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C3" s="5">
         <v>46068</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="G3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="I3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="6" t="s">
-        <v>19</v>
-      </c>
       <c r="J3" s="6" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>21</v>
+        <v>199</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>22</v>
+        <v>200</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="N3" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="4" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="4" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A4" s="3">
         <v>7</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C4" s="5">
         <v>46068</v>
       </c>
       <c r="D4" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="H4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="G4" s="6" t="s">
+      <c r="I4" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="J4" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="H4" s="17" t="s">
-        <v>234</v>
-      </c>
-      <c r="I4" s="17" t="s">
-        <v>225</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>33</v>
-      </c>
       <c r="K4" s="6" t="s">
-        <v>34</v>
+        <v>201</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>35</v>
+        <v>202</v>
       </c>
       <c r="M4" s="6"/>
       <c r="N4" s="3">
         <v>1555</v>
       </c>
     </row>
-    <row r="5" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="5" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A5" s="3">
         <v>8</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C5" s="5">
         <v>46068</v>
       </c>
       <c r="D5" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="F5" s="6" t="s">
+      <c r="I5" s="17" t="s">
+        <v>191</v>
+      </c>
+      <c r="J5" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="G5" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="I5" s="17" t="s">
-        <v>226</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>43</v>
-      </c>
       <c r="K5" s="6" t="s">
-        <v>44</v>
+        <v>204</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>45</v>
+        <v>205</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="N5" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="6" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="6" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A6" s="3">
         <v>9</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C6" s="5">
         <v>46068</v>
       </c>
-      <c r="D6" s="6" t="s">
-        <v>47</v>
+      <c r="D6" s="17" t="s">
+        <v>203</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="I6" s="17" t="s">
-        <v>226</v>
+        <v>37</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>38</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>44</v>
+        <v>204</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>45</v>
+        <v>205</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="N6" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="7" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="7" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A7" s="3">
         <v>10</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="C7" s="5">
         <v>46068</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>34</v>
+        <v>201</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>35</v>
+        <v>202</v>
       </c>
       <c r="M7" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N7" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="8" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="8" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A8" s="3">
         <v>11</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C8" s="5">
         <v>46068</v>
       </c>
       <c r="D8" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="J8" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E8" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>58</v>
-      </c>
       <c r="K8" s="6" t="s">
-        <v>34</v>
+        <v>201</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>35</v>
+        <v>202</v>
       </c>
       <c r="M8" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N8" s="3">
         <v>1532</v>
@@ -3387,126 +3170,126 @@
         <v>13</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="C9" s="5">
         <v>46068</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>231</v>
+        <v>196</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>63</v>
+        <v>55</v>
+      </c>
+      <c r="I9" s="17" t="s">
+        <v>236</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>65</v>
+        <v>206</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>66</v>
+        <v>207</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="N9" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="10" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="10" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A10" s="3">
         <v>15</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C10" s="5">
         <v>46068</v>
       </c>
-      <c r="D10" s="6" t="s">
-        <v>68</v>
+      <c r="D10" s="17" t="s">
+        <v>231</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="I10" s="17" t="s">
-        <v>227</v>
+        <v>192</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>73</v>
+        <v>208</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>74</v>
+        <v>209</v>
       </c>
       <c r="M10" s="6"/>
       <c r="N10" s="3">
         <v>1534</v>
       </c>
     </row>
-    <row r="11" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="11" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A11" s="3">
         <v>18</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="C11" s="5">
         <v>46068</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>76</v>
+      <c r="D11" s="17" t="s">
+        <v>233</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>34</v>
+        <v>201</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>35</v>
+        <v>202</v>
       </c>
       <c r="M11" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N11" s="3">
         <v>1532</v>
@@ -3517,442 +3300,442 @@
         <v>20</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="C12" s="5">
         <v>46068</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>63</v>
+        <v>55</v>
+      </c>
+      <c r="I12" s="17" t="s">
+        <v>236</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>65</v>
+        <v>206</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>66</v>
+        <v>207</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="N12" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="13" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="13" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A13" s="3">
         <v>23</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="C13" s="5">
         <v>46068</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="E13" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="I13" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="F13" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>42</v>
-      </c>
       <c r="J13" s="6" t="s">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>89</v>
+        <v>210</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>22</v>
+        <v>200</v>
       </c>
       <c r="M13" s="4" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="N13" s="3">
         <v>506</v>
       </c>
     </row>
-    <row r="14" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="14" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A14" s="3">
         <v>24</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="C14" s="5">
         <v>46068</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>228</v>
+        <v>193</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>89</v>
+        <v>210</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>22</v>
+        <v>200</v>
       </c>
       <c r="M14" s="4" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="N14" s="3">
         <v>506</v>
       </c>
     </row>
-    <row r="15" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="15" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A15" s="3">
         <v>25</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="C15" s="5">
         <v>46068</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>21</v>
+        <v>199</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="N15" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="16" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="16" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A16" s="3">
         <v>26</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="C16" s="5">
         <v>46068</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="H16" s="10" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>21</v>
+        <v>199</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="M16" s="10" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="N16" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="17" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="17" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A17" s="3">
         <v>28</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="C17" s="5">
         <v>46068</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="E17" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="H17" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="I17" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="F17" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="H17" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>42</v>
-      </c>
       <c r="J17" s="6" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>107</v>
+        <v>212</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>108</v>
+        <v>213</v>
       </c>
       <c r="M17" s="11" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="N17" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="18" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="18" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A18" s="3">
         <v>29</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>109</v>
+        <v>92</v>
       </c>
       <c r="C18" s="5">
         <v>46068</v>
       </c>
       <c r="D18" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J18" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="E18" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="H18" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="I18" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="J18" s="6" t="s">
-        <v>111</v>
-      </c>
       <c r="K18" s="6" t="s">
-        <v>107</v>
+        <v>212</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>108</v>
+        <v>213</v>
       </c>
       <c r="M18" s="11" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="N18" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="19" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="19" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A19" s="3">
         <v>32</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="C19" s="5">
         <v>46068</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>118</v>
+        <v>101</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>119</v>
+        <v>214</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>120</v>
+        <v>215</v>
       </c>
       <c r="M19" s="12" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="N19" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="20" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="20" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A20" s="3">
         <v>33</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>121</v>
+        <v>102</v>
       </c>
       <c r="C20" s="5">
         <v>46068</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>122</v>
+        <v>103</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>119</v>
+        <v>214</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>120</v>
+        <v>215</v>
       </c>
       <c r="M20" s="12" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="N20" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="21" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="21" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A21" s="3">
         <v>37</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="C21" s="5">
         <v>46068</v>
       </c>
-      <c r="D21" s="6" t="s">
-        <v>125</v>
+      <c r="D21" s="17" t="s">
+        <v>194</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>126</v>
+        <v>106</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>34</v>
+        <v>201</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>35</v>
+        <v>202</v>
       </c>
       <c r="M21" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N21" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="22" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="22" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A22" s="3">
         <v>41</v>
       </c>
@@ -3960,167 +3743,167 @@
       <c r="C22" s="5">
         <v>46068</v>
       </c>
-      <c r="D22" s="6" t="s">
-        <v>127</v>
+      <c r="D22" s="17" t="s">
+        <v>226</v>
       </c>
       <c r="E22" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="I22" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="F22" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="G22" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="H22" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="I22" s="6" t="s">
-        <v>42</v>
-      </c>
       <c r="J22" s="6" t="s">
-        <v>129</v>
+        <v>108</v>
       </c>
       <c r="K22" s="6" t="s">
-        <v>89</v>
+        <v>210</v>
       </c>
       <c r="L22" s="6" t="s">
-        <v>22</v>
+        <v>200</v>
       </c>
       <c r="M22" s="4" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="N22" s="3">
         <v>506</v>
       </c>
     </row>
-    <row r="23" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="23" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A23" s="3">
         <v>42</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>130</v>
+        <v>109</v>
       </c>
       <c r="C23" s="5">
         <v>46068</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>229</v>
+        <v>194</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="H23" s="12" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>222</v>
+        <v>187</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>132</v>
+        <v>111</v>
       </c>
       <c r="K23" s="6" t="s">
-        <v>133</v>
+        <v>216</v>
       </c>
       <c r="L23" s="6" t="s">
-        <v>134</v>
+        <v>217</v>
       </c>
       <c r="M23" s="12" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="N23" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="24" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="24" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A24" s="3">
         <v>43</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>135</v>
+        <v>112</v>
       </c>
       <c r="C24" s="5">
         <v>46068</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>136</v>
+        <v>113</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>137</v>
+        <v>114</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>223</v>
+        <v>188</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>138</v>
+        <v>115</v>
       </c>
       <c r="K24" s="6" t="s">
-        <v>139</v>
+        <v>218</v>
       </c>
       <c r="L24" s="6" t="s">
-        <v>140</v>
+        <v>219</v>
       </c>
       <c r="M24" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N24" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="25" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="25" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A25" s="3">
         <v>44</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>141</v>
+        <v>116</v>
       </c>
       <c r="C25" s="5">
         <v>46068</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>136</v>
+        <v>113</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>142</v>
+        <v>117</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>223</v>
+        <v>188</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>143</v>
+        <v>118</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>139</v>
+        <v>218</v>
       </c>
       <c r="L25" s="6" t="s">
-        <v>140</v>
+        <v>219</v>
       </c>
       <c r="M25" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N25" s="3">
         <v>1532</v>
@@ -4131,871 +3914,882 @@
         <v>46</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>144</v>
+        <v>119</v>
       </c>
       <c r="C26" s="5">
         <v>46068</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>145</v>
+        <v>120</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>146</v>
+        <v>121</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="I26" s="4" t="s">
-        <v>63</v>
+        <v>122</v>
+      </c>
+      <c r="I26" s="17" t="s">
+        <v>236</v>
       </c>
       <c r="J26" s="6" t="s">
-        <v>148</v>
+        <v>123</v>
       </c>
       <c r="K26" s="6" t="s">
-        <v>65</v>
+        <v>206</v>
       </c>
       <c r="L26" s="6" t="s">
-        <v>66</v>
+        <v>207</v>
       </c>
       <c r="M26" s="6"/>
       <c r="N26" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="27" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="27" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A27" s="3">
         <v>47</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>149</v>
+        <v>124</v>
       </c>
       <c r="C27" s="5">
         <v>46068</v>
       </c>
       <c r="D27" s="17" t="s">
-        <v>232</v>
+        <v>197</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>151</v>
+        <v>126</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>152</v>
+        <v>127</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>153</v>
+        <v>128</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>154</v>
+        <v>129</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>21</v>
+        <v>199</v>
       </c>
       <c r="L27" s="6" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="M27" s="6"/>
       <c r="N27" s="3">
         <v>1534</v>
       </c>
     </row>
-    <row r="28" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="28" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A28" s="3">
         <v>48</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>155</v>
+        <v>130</v>
       </c>
       <c r="C28" s="5">
         <v>46068</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>150</v>
+        <v>125</v>
       </c>
       <c r="E28" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F28" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="F28" s="6" t="s">
-        <v>156</v>
-      </c>
       <c r="G28" s="6" t="s">
-        <v>157</v>
+        <v>132</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>158</v>
+        <v>133</v>
       </c>
       <c r="I28" s="17" t="s">
-        <v>224</v>
+        <v>189</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>159</v>
+        <v>134</v>
       </c>
       <c r="K28" s="6" t="s">
-        <v>160</v>
+        <v>220</v>
       </c>
       <c r="L28" s="6" t="s">
-        <v>161</v>
+        <v>221</v>
       </c>
       <c r="M28" s="6"/>
       <c r="N28" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="29" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="29" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A29" s="3">
         <v>52</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>162</v>
+        <v>135</v>
       </c>
       <c r="C29" s="5">
         <v>46068</v>
       </c>
       <c r="D29" s="17" t="s">
-        <v>230</v>
+        <v>195</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>163</v>
+        <v>136</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>164</v>
+        <v>137</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>165</v>
+        <v>138</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>166</v>
+        <v>139</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="K29" s="4"/>
+        <v>140</v>
+      </c>
+      <c r="K29" s="6" t="s">
+        <v>139</v>
+      </c>
       <c r="L29" s="6" t="s">
-        <v>134</v>
+        <v>217</v>
       </c>
       <c r="M29" s="6"/>
       <c r="N29" s="3">
         <v>1535</v>
       </c>
     </row>
-    <row r="30" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="30" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A30" s="3">
         <v>53</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>168</v>
+        <v>141</v>
       </c>
       <c r="C30" s="5">
         <v>46068</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>169</v>
+        <v>142</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>170</v>
+        <v>143</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J30" s="6" t="s">
-        <v>171</v>
+        <v>144</v>
       </c>
       <c r="K30" s="6" t="s">
-        <v>34</v>
+        <v>201</v>
       </c>
       <c r="L30" s="6" t="s">
-        <v>35</v>
+        <v>202</v>
       </c>
       <c r="M30" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N30" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="31" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="31" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A31" s="3">
         <v>54</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>172</v>
+        <v>145</v>
       </c>
       <c r="C31" s="5">
         <v>46068</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>169</v>
+        <v>142</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>170</v>
+        <v>143</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J31" s="6" t="s">
-        <v>173</v>
+        <v>146</v>
       </c>
       <c r="K31" s="6" t="s">
-        <v>34</v>
+        <v>201</v>
       </c>
       <c r="L31" s="6" t="s">
-        <v>35</v>
+        <v>202</v>
       </c>
       <c r="M31" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N31" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="32" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="32" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A32" s="3">
         <v>55</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>174</v>
+        <v>147</v>
       </c>
       <c r="C32" s="5">
         <v>46068</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>175</v>
+        <v>148</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>176</v>
+        <v>149</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>137</v>
+        <v>114</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>223</v>
+        <v>188</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>177</v>
+        <v>150</v>
       </c>
       <c r="K32" s="6" t="s">
-        <v>139</v>
+        <v>218</v>
       </c>
       <c r="L32" s="6" t="s">
-        <v>140</v>
+        <v>219</v>
       </c>
       <c r="M32" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N32" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="33" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="33" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A33" s="3">
         <v>56</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>178</v>
+        <v>151</v>
       </c>
       <c r="C33" s="5">
         <v>46068</v>
       </c>
-      <c r="D33" s="6" t="s">
-        <v>179</v>
+      <c r="D33" s="17" t="s">
+        <v>234</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>170</v>
+        <v>143</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>223</v>
+        <v>188</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>180</v>
+        <v>152</v>
       </c>
       <c r="K33" s="6" t="s">
-        <v>139</v>
+        <v>218</v>
       </c>
       <c r="L33" s="6" t="s">
-        <v>140</v>
+        <v>219</v>
       </c>
       <c r="M33" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N33" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="34" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="34" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A34" s="3">
         <v>57</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>181</v>
+        <v>153</v>
       </c>
       <c r="C34" s="5">
         <v>46068</v>
       </c>
-      <c r="D34" s="6" t="s">
-        <v>182</v>
+      <c r="D34" s="17" t="s">
+        <v>222</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>183</v>
+        <v>154</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="H34" s="7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>184</v>
+        <v>155</v>
       </c>
       <c r="K34" s="6" t="s">
-        <v>44</v>
+        <v>204</v>
       </c>
       <c r="L34" s="6" t="s">
-        <v>45</v>
+        <v>205</v>
       </c>
       <c r="M34" s="7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="N34" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="35" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="35" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A35" s="3">
         <v>60</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>185</v>
+        <v>156</v>
       </c>
       <c r="C35" s="5">
         <v>46068</v>
       </c>
-      <c r="D35" s="6" t="s">
-        <v>186</v>
+      <c r="D35" s="17" t="s">
+        <v>230</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>187</v>
+        <v>157</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="H35" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I35" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="I35" s="6" t="s">
-        <v>19</v>
-      </c>
       <c r="J35" s="6" t="s">
-        <v>188</v>
+        <v>158</v>
       </c>
       <c r="K35" s="6" t="s">
-        <v>21</v>
+        <v>199</v>
       </c>
       <c r="L35" s="6" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="M35" s="6"/>
       <c r="N35" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="36" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="36" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A36" s="3">
         <v>62</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>189</v>
+        <v>159</v>
       </c>
       <c r="C36" s="5">
         <v>46068</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>190</v>
+        <v>160</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>191</v>
+        <v>161</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>192</v>
+        <v>162</v>
       </c>
       <c r="H36" s="14" t="s">
-        <v>193</v>
+        <v>163</v>
       </c>
       <c r="I36" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>194</v>
+        <v>164</v>
       </c>
       <c r="K36" s="6" t="s">
-        <v>195</v>
+        <v>223</v>
       </c>
       <c r="L36" s="6" t="s">
-        <v>161</v>
+        <v>221</v>
       </c>
       <c r="M36" s="14" t="s">
-        <v>193</v>
+        <v>163</v>
       </c>
       <c r="N36" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="37" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="37" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A37" s="3">
         <v>63</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>196</v>
+        <v>165</v>
       </c>
       <c r="C37" s="5">
         <v>46068</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>190</v>
+        <v>160</v>
       </c>
       <c r="E37" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F37" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F37" s="6" t="s">
-        <v>16</v>
-      </c>
       <c r="G37" s="6" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="H37" s="12" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>197</v>
+        <v>166</v>
       </c>
       <c r="K37" s="6" t="s">
-        <v>119</v>
+        <v>214</v>
       </c>
       <c r="L37" s="6" t="s">
-        <v>120</v>
+        <v>215</v>
       </c>
       <c r="M37" s="12" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="N37" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="38" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="38" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A38" s="3">
         <v>64</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>198</v>
+        <v>167</v>
       </c>
       <c r="C38" s="5">
         <v>46068</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>199</v>
+        <v>168</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>200</v>
+        <v>169</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="H38" s="12" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="I38" s="6" t="s">
-        <v>222</v>
+        <v>187</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>201</v>
+        <v>170</v>
       </c>
       <c r="K38" s="6" t="s">
-        <v>133</v>
+        <v>216</v>
       </c>
       <c r="L38" s="6" t="s">
-        <v>134</v>
+        <v>217</v>
       </c>
       <c r="M38" s="12" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="N38" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="39" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="39" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A39" s="3">
         <v>69</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>202</v>
+        <v>171</v>
       </c>
       <c r="C39" s="5">
         <v>46068</v>
       </c>
-      <c r="D39" s="6" t="s">
-        <v>203</v>
+      <c r="D39" s="17" t="s">
+        <v>232</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>170</v>
+        <v>143</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>142</v>
+        <v>117</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="H39" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
       <c r="K39" s="6" t="s">
-        <v>205</v>
+        <v>224</v>
       </c>
       <c r="L39" s="6" t="s">
-        <v>140</v>
+        <v>219</v>
       </c>
       <c r="M39" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N39" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="40" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="40" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A40" s="3">
         <v>73</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>206</v>
+        <v>173</v>
       </c>
       <c r="C40" s="5">
         <v>46068</v>
       </c>
-      <c r="D40" s="6" t="s">
-        <v>203</v>
+      <c r="D40" s="17" t="s">
+        <v>235</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>207</v>
+        <v>174</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="H40" s="11" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="I40" s="6" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J40" s="6" t="s">
-        <v>208</v>
+        <v>175</v>
       </c>
       <c r="K40" s="6" t="s">
-        <v>107</v>
+        <v>212</v>
       </c>
       <c r="L40" s="6" t="s">
-        <v>108</v>
+        <v>213</v>
       </c>
       <c r="M40" s="11" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="N40" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="41" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="41" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A41" s="3">
         <v>76</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>209</v>
+        <v>176</v>
       </c>
       <c r="C41" s="5">
         <v>46068</v>
       </c>
-      <c r="D41" s="6" t="s">
-        <v>210</v>
+      <c r="D41" s="17" t="s">
+        <v>229</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>211</v>
+        <v>177</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>212</v>
+        <v>178</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>213</v>
+        <v>179</v>
       </c>
       <c r="H41" s="14" t="s">
-        <v>193</v>
+        <v>163</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>208</v>
+        <v>175</v>
       </c>
       <c r="K41" s="6" t="s">
-        <v>195</v>
+        <v>223</v>
       </c>
       <c r="L41" s="6" t="s">
-        <v>161</v>
+        <v>221</v>
       </c>
       <c r="M41" s="14" t="s">
-        <v>193</v>
+        <v>163</v>
       </c>
       <c r="N41" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="42" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="42" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A42" s="3">
         <v>83</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>214</v>
+        <v>180</v>
       </c>
       <c r="C42" s="5">
         <v>46068</v>
       </c>
-      <c r="D42" s="6" t="s">
-        <v>210</v>
+      <c r="D42" s="17" t="s">
+        <v>227</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>215</v>
+        <v>181</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="H42" s="12" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="I42" s="6" t="s">
-        <v>222</v>
+        <v>187</v>
       </c>
       <c r="J42" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="K42" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="K42" s="6" t="s">
-        <v>133</v>
-      </c>
       <c r="L42" s="6" t="s">
-        <v>134</v>
+        <v>217</v>
       </c>
       <c r="M42" s="12" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="N42" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="43" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="43" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A43" s="3">
         <v>84</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>217</v>
+        <v>183</v>
       </c>
       <c r="C43" s="5">
         <v>46068</v>
       </c>
-      <c r="D43" s="6" t="s">
-        <v>210</v>
+      <c r="D43" s="17" t="s">
+        <v>225</v>
       </c>
       <c r="E43" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="G43" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="H43" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="I43" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="J43" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="K43" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="L43" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="F43" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="G43" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="H43" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="I43" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="J43" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="K43" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="L43" s="6" t="s">
-        <v>120</v>
-      </c>
       <c r="M43" s="12" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="N43" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="44" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="44" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A44" s="3">
         <v>85</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>219</v>
+        <v>185</v>
       </c>
       <c r="C44" s="5">
         <v>46068</v>
       </c>
-      <c r="D44" s="6" t="s">
-        <v>210</v>
+      <c r="D44" s="17" t="s">
+        <v>225</v>
       </c>
       <c r="E44" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="F44" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G44" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="H44" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="I44" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="J44" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="K44" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="L44" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="F44" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="G44" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="H44" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="I44" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="J44" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="K44" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="L44" s="6" t="s">
-        <v>120</v>
-      </c>
       <c r="M44" s="12" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="N44" s="3">
         <v>1532</v>
       </c>
     </row>
-    <row r="45" spans="1:14" s="2" customFormat="1" ht="32.25" customHeight="1">
+    <row r="45" spans="1:14" s="2" customFormat="1" ht="32.25" hidden="1" customHeight="1">
       <c r="A45" s="3">
         <v>86</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>220</v>
+        <v>186</v>
       </c>
       <c r="C45" s="5">
         <v>46068</v>
       </c>
-      <c r="D45" s="6" t="s">
-        <v>210</v>
+      <c r="D45" s="17" t="s">
+        <v>227</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>215</v>
+        <v>181</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="G45" s="6" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="H45" s="12" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="I45" s="6" t="s">
-        <v>222</v>
+        <v>187</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>132</v>
+        <v>111</v>
       </c>
       <c r="K45" s="6" t="s">
-        <v>133</v>
+        <v>216</v>
       </c>
       <c r="L45" s="6" t="s">
-        <v>134</v>
+        <v>217</v>
       </c>
       <c r="M45" s="12" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="N45" s="3">
         <v>1532</v>
       </c>
     </row>
+    <row r="47" spans="1:14">
+      <c r="D47" s="18"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N45" xr:uid="{A581A1F3-CAF0-45C6-9B1F-97A2BD6208C7}"/>
+  <autoFilter ref="A1:N45" xr:uid="{A581A1F3-CAF0-45C6-9B1F-97A2BD6208C7}">
+    <filterColumn colId="8">
+      <filters>
+        <filter val="4.2 Ton Double cabin Open Truck_x000a_(with lift)"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>